<commit_message>
Refresh comparison harness results for the new library set
Update Results.xlsx (raw data, pivot cache, and pivot chart) to replace the
retired SharpDX benchmark with System.Numerics and refresh all timings from a
fresh run. The pivot cache is set to refresh on load so the chart redraws when
the workbook is opened.
</commit_message>
<xml_diff>
--- a/RP.Math.Vector3.ComparisonHarness/Results.xlsx
+++ b/RP.Math.Vector3.ComparisonHarness/Results.xlsx
@@ -51,7 +51,7 @@
     <t xml:space="preserve"> MathNet</t>
   </si>
   <si>
-    <t xml:space="preserve"> SharpDX</t>
+    <t xml:space="preserve"> System.Numerics</t>
   </si>
   <si>
     <t xml:space="preserve"> Seven</t>
@@ -664,19 +664,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2178</c:v>
+                  <c:v>925</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2530</c:v>
+                  <c:v>1812</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1937</c:v>
+                  <c:v>887</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3347</c:v>
+                  <c:v>1977</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2461</c:v>
+                  <c:v>930</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -795,19 +795,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>25093</c:v>
+                  <c:v>8331</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>155219</c:v>
+                  <c:v>82992</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7240</c:v>
+                  <c:v>3599</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>53003</c:v>
+                  <c:v>29345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13901</c:v>
+                  <c:v>22337</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -928,19 +928,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3980</c:v>
+                  <c:v>1306</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8989</c:v>
+                  <c:v>2311</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4670</c:v>
+                  <c:v>1425</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>16959</c:v>
+                  <c:v>7024</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3464</c:v>
+                  <c:v>1267</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1059,19 +1059,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9933</c:v>
+                  <c:v>3991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11943</c:v>
+                  <c:v>6100</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7250</c:v>
+                  <c:v>3167</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>68515</c:v>
+                  <c:v>6108</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9599</c:v>
+                  <c:v>4241</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1086,7 +1086,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v> SharpDX</c:v>
+                  <c:v> System.Numerics</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1190,19 +1190,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2128</c:v>
+                  <c:v>635</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3175</c:v>
+                  <c:v>721</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1867</c:v>
+                  <c:v>707</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4429</c:v>
+                  <c:v>784</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2000</c:v>
+                  <c:v>466</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2129,7 +2129,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="richard Potter" refreshedDate="42026.390067939814" createdVersion="5" refreshedVersion="5" minRefreshableVersion="3" recordCount="25">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" r:id="rId1" refreshedBy="richard Potter" refreshedDate="42026.390067939814" createdVersion="5" refreshedVersion="5" minRefreshableVersion="3" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource name="Table1"/>
   </cacheSource>
@@ -2138,7 +2138,7 @@
       <sharedItems count="5">
         <s v=" RP.Math.Vector3"/>
         <s v=" MathNet"/>
-        <s v=" SharpDX"/>
+        <s v=" System.Numerics"/>
         <s v=" Seven"/>
         <s v=" Exocortex"/>
       </sharedItems>
@@ -2153,7 +2153,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Time" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1867" maxValue="155219"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="466" maxValue="82992"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -2169,127 +2169,127 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="8989"/>
+    <n v="2311"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="4670"/>
+    <n v="1425"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <n v="16959"/>
+    <n v="7024"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <n v="3980"/>
+    <n v="1306"/>
   </r>
   <r>
     <x v="0"/>
     <x v="4"/>
-    <n v="3464"/>
+    <n v="1267"/>
   </r>
   <r>
     <x v="1"/>
     <x v="0"/>
-    <n v="155219"/>
+    <n v="82992"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
-    <n v="7240"/>
+    <n v="3599"/>
   </r>
   <r>
     <x v="1"/>
     <x v="2"/>
-    <n v="53003"/>
+    <n v="29345"/>
   </r>
   <r>
     <x v="1"/>
     <x v="3"/>
-    <n v="25093"/>
+    <n v="8331"/>
   </r>
   <r>
     <x v="1"/>
     <x v="4"/>
-    <n v="13901"/>
+    <n v="22337"/>
   </r>
   <r>
     <x v="2"/>
     <x v="0"/>
-    <n v="3175"/>
+    <n v="721"/>
   </r>
   <r>
     <x v="2"/>
     <x v="1"/>
-    <n v="1867"/>
+    <n v="707"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
-    <n v="4429"/>
+    <n v="784"/>
   </r>
   <r>
     <x v="2"/>
     <x v="3"/>
-    <n v="2128"/>
+    <n v="635"/>
   </r>
   <r>
     <x v="2"/>
     <x v="4"/>
-    <n v="2000"/>
+    <n v="466"/>
   </r>
   <r>
     <x v="3"/>
     <x v="0"/>
-    <n v="11943"/>
+    <n v="6100"/>
   </r>
   <r>
     <x v="3"/>
     <x v="1"/>
-    <n v="7250"/>
+    <n v="3167"/>
   </r>
   <r>
     <x v="3"/>
     <x v="2"/>
-    <n v="68515"/>
+    <n v="6108"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
-    <n v="9933"/>
+    <n v="3991"/>
   </r>
   <r>
     <x v="3"/>
     <x v="4"/>
-    <n v="9599"/>
+    <n v="4241"/>
   </r>
   <r>
     <x v="4"/>
     <x v="0"/>
-    <n v="2530"/>
+    <n v="1812"/>
   </r>
   <r>
     <x v="4"/>
     <x v="1"/>
-    <n v="1937"/>
+    <n v="887"/>
   </r>
   <r>
     <x v="4"/>
     <x v="2"/>
-    <n v="3347"/>
+    <n v="1977"/>
   </r>
   <r>
     <x v="4"/>
     <x v="3"/>
-    <n v="2178"/>
+    <n v="925"/>
   </r>
   <r>
     <x v="4"/>
     <x v="4"/>
-    <n v="2461"/>
+    <n v="930"/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>8989</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2951,7 +2951,7 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>4670</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2962,7 +2962,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>16959</v>
+        <v>7024</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2973,7 +2973,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>3980</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2984,7 +2984,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>3464</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2995,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>155219</v>
+        <v>82992</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3006,7 +3006,7 @@
         <v>2</v>
       </c>
       <c r="C8">
-        <v>7240</v>
+        <v>3599</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3017,7 +3017,7 @@
         <v>3</v>
       </c>
       <c r="C9">
-        <v>53003</v>
+        <v>29345</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3028,7 +3028,7 @@
         <v>4</v>
       </c>
       <c r="C10">
-        <v>25093</v>
+        <v>8331</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3039,7 +3039,7 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>13901</v>
+        <v>22337</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3050,7 +3050,7 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>3175</v>
+        <v>721</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3061,7 +3061,7 @@
         <v>2</v>
       </c>
       <c r="C13">
-        <v>1867</v>
+        <v>707</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3072,7 +3072,7 @@
         <v>3</v>
       </c>
       <c r="C14">
-        <v>4429</v>
+        <v>784</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3083,7 +3083,7 @@
         <v>4</v>
       </c>
       <c r="C15">
-        <v>2128</v>
+        <v>635</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3094,7 +3094,7 @@
         <v>5</v>
       </c>
       <c r="C16">
-        <v>2000</v>
+        <v>466</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3105,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="C17">
-        <v>11943</v>
+        <v>6100</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3116,7 +3116,7 @@
         <v>2</v>
       </c>
       <c r="C18">
-        <v>7250</v>
+        <v>3167</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -3127,7 +3127,7 @@
         <v>3</v>
       </c>
       <c r="C19">
-        <v>68515</v>
+        <v>6108</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -3138,7 +3138,7 @@
         <v>4</v>
       </c>
       <c r="C20">
-        <v>9933</v>
+        <v>3991</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -3149,7 +3149,7 @@
         <v>5</v>
       </c>
       <c r="C21">
-        <v>9599</v>
+        <v>4241</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -3160,7 +3160,7 @@
         <v>0</v>
       </c>
       <c r="C22">
-        <v>2530</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -3171,7 +3171,7 @@
         <v>2</v>
       </c>
       <c r="C23">
-        <v>1937</v>
+        <v>887</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -3182,7 +3182,7 @@
         <v>3</v>
       </c>
       <c r="C24">
-        <v>3347</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3193,7 +3193,7 @@
         <v>4</v>
       </c>
       <c r="C25">
-        <v>2178</v>
+        <v>925</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3204,7 +3204,7 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>2461</v>
+        <v>930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>